<commit_message>
Synchronize latest local snapshot
</commit_message>
<xml_diff>
--- a/Boltonia_all_metadata_20251010.xlsx
+++ b/Boltonia_all_metadata_20251010.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gowustl-my.sharepoint.com/personal/wen-hsi_kuo_wustl_edu/Documents/MOBOT/MOBOT_Boltonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_9C3C1DD08F79A823E4237872E07BD272CA4AEB63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22BBB160-AA99-0649-9C16-AA5520D83297}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_9C3C1DD08F79A823E4237872E07BD272CA4AEB63" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{908472C2-1D4E-9241-B7B5-44FD7C82EA37}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="500" windowWidth="43880" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2686,6 +2686,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="18" max="18" width="62.33203125" customWidth="1"/>
     <col min="19" max="20" width="20.6640625" style="2" customWidth="1"/>
     <col min="21" max="21" width="20.6640625" style="3" customWidth="1"/>
     <col min="26" max="26" width="20.6640625" style="2" customWidth="1"/>

</xml_diff>